<commit_message>
Fix: FRACAS yazma hatası - hourly_rate ve personnel_count float türüne dönüştürüldü
</commit_message>
<xml_diff>
--- a/data/kocaeli/Veriler.xlsx
+++ b/data/kocaeli/Veriler.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fatiherkin\Desktop\bozankaya_ssh_takip\data\kocaeli\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F84FEBA1-EFF7-4BFC-B8A0-BF500D399DE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7844EDDC-B026-4A43-AD8D-4F905FB6576E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="201">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="204">
   <si>
     <t>Traction_Converter</t>
   </si>
@@ -96,9 +96,6 @@
     <t>Cab_Desk</t>
   </si>
   <si>
-    <t>Cable_Duct</t>
-  </si>
-  <si>
     <t>CCTV</t>
   </si>
   <si>
@@ -126,9 +123,6 @@
     <t>Light_Barrier</t>
   </si>
   <si>
-    <t>Horn_Bell</t>
-  </si>
-  <si>
     <t>Wiper_System</t>
   </si>
   <si>
@@ -162,45 +156,21 @@
     <t>Medcom</t>
   </si>
   <si>
-    <t>HBL</t>
-  </si>
-  <si>
     <t>Bozankaya</t>
   </si>
   <si>
-    <t>MİNEL</t>
-  </si>
-  <si>
     <t>Secheron</t>
   </si>
   <si>
     <t>ALFA UNİON</t>
   </si>
   <si>
-    <t>Wicov</t>
-  </si>
-  <si>
     <t>A</t>
   </si>
   <si>
-    <t>Hanning&amp;Kall</t>
-  </si>
-  <si>
     <t>SKF</t>
   </si>
   <si>
-    <t>HISPACOLD</t>
-  </si>
-  <si>
-    <t>G</t>
-  </si>
-  <si>
-    <t>BOZANKAYA</t>
-  </si>
-  <si>
-    <t>NOVATRONİK</t>
-  </si>
-  <si>
     <t>ERA</t>
   </si>
   <si>
@@ -213,9 +183,6 @@
     <t>Alfa UNION</t>
   </si>
   <si>
-    <t>PSV</t>
-  </si>
-  <si>
     <t>Hanning&amp;Kahl</t>
   </si>
   <si>
@@ -585,9 +552,6 @@
     <t>Arıza Tipi</t>
   </si>
   <si>
-    <t>MC</t>
-  </si>
-  <si>
     <t>A-Kritik/Emniyet Riski</t>
   </si>
   <si>
@@ -597,9 +561,6 @@
     <t>KOCAELİ</t>
   </si>
   <si>
-    <t>SA</t>
-  </si>
-  <si>
     <t>B-Yüksek/Operasyon Engeller</t>
   </si>
   <si>
@@ -609,9 +570,6 @@
     <t>(II) Aynı Araçta Tekrarlayan Arıza</t>
   </si>
   <si>
-    <t>T</t>
-  </si>
-  <si>
     <t>C-Hafif/Kısıtlı Operasyon</t>
   </si>
   <si>
@@ -621,15 +579,9 @@
     <t>(III) Farklı Araçlarda Tekrarlayan Arıza</t>
   </si>
   <si>
-    <t>SB</t>
-  </si>
-  <si>
     <t>D-Arıza Değildir</t>
   </si>
   <si>
-    <t>M</t>
-  </si>
-  <si>
     <t>KOC10</t>
   </si>
   <si>
@@ -637,6 +589,63 @@
   </si>
   <si>
     <t xml:space="preserve"> £11,00 </t>
+  </si>
+  <si>
+    <t>MA</t>
+  </si>
+  <si>
+    <t>MB</t>
+  </si>
+  <si>
+    <t>RA</t>
+  </si>
+  <si>
+    <t>P</t>
+  </si>
+  <si>
+    <t>RB</t>
+  </si>
+  <si>
+    <t>ASİPLSAN</t>
+  </si>
+  <si>
+    <t>SCHUNK</t>
+  </si>
+  <si>
+    <t>IGW</t>
+  </si>
+  <si>
+    <t>KNOR BREMSE</t>
+  </si>
+  <si>
+    <t>KAAF</t>
+  </si>
+  <si>
+    <t>ELTESAN</t>
+  </si>
+  <si>
+    <t>ATAK ULAŞIM</t>
+  </si>
+  <si>
+    <t>DELLNER</t>
+  </si>
+  <si>
+    <t>DENİZLER</t>
+  </si>
+  <si>
+    <t>HORN</t>
+  </si>
+  <si>
+    <t>BOSCH</t>
+  </si>
+  <si>
+    <t>Bell</t>
+  </si>
+  <si>
+    <t>ASELSAN</t>
+  </si>
+  <si>
+    <t>ISRI</t>
   </si>
 </sst>
 </file>
@@ -693,7 +702,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -710,12 +719,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
     <fill>
@@ -803,7 +806,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -824,31 +827,28 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -1251,1081 +1251,1085 @@
         <v>19</v>
       </c>
       <c r="U1" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="V1" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="2" t="s">
+      <c r="W1" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="2" t="s">
+      <c r="X1" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="2" t="s">
+      <c r="Y1" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="2" t="s">
+      <c r="Z1" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="2" t="s">
+      <c r="AA1" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="2" t="s">
+      <c r="AB1" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="AB1" s="2" t="s">
+      <c r="AC1" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="AC1" s="2" t="s">
+      <c r="AD1" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="AD1" s="2" t="s">
+      <c r="AE1" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="AF1" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="AE1" s="2" t="s">
+      <c r="AG1" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="AF1" s="2" t="s">
+      <c r="AH1" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="AG1" s="2" t="s">
+      <c r="AI1" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="AH1" s="2" t="s">
+      <c r="AJ1" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="AI1" s="2" t="s">
+      <c r="AK1" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="AJ1" s="2" t="s">
+      <c r="AL1" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="AK1" s="2" t="s">
+      <c r="AM1" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="AL1" s="2" t="s">
+      <c r="AN1" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="AM1" s="2" t="s">
+      <c r="AO1" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="AN1" s="2" t="s">
+    </row>
+    <row r="2" spans="1:41" ht="19.2" x14ac:dyDescent="0.3">
+      <c r="A2" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="AO1" s="3" t="s">
+      <c r="B2" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>190</v>
+      </c>
+      <c r="D2" s="5" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="2" spans="1:41" x14ac:dyDescent="0.3">
-      <c r="A2" s="4" t="s">
+      <c r="E2" s="5" t="s">
+        <v>191</v>
+      </c>
+      <c r="F2" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="B2" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="C2" s="5" t="s">
+      <c r="G2" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="H2" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="I2" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="J2" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="K2" s="6" t="s">
+        <v>192</v>
+      </c>
+      <c r="L2" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="M2" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="N2" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="O2" s="5" t="s">
+        <v>194</v>
+      </c>
+      <c r="P2" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q2" s="6" t="s">
+        <v>195</v>
+      </c>
+      <c r="R2" s="6" t="s">
+        <v>195</v>
+      </c>
+      <c r="S2" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="T2" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="U2" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="V2" s="5" t="s">
+        <v>196</v>
+      </c>
+      <c r="W2" s="5" t="s">
+        <v>196</v>
+      </c>
+      <c r="X2" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="G2" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="H2" s="5" t="s">
+      <c r="Y2" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z2" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="I2" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="J2" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="K2" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="L2" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="M2" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="N2" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="O2" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="P2" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="Q2" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="R2" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="S2" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="T2" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="U2" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="V2" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="W2" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="X2" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="Y2" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="Z2" s="6" t="s">
-        <v>56</v>
-      </c>
       <c r="AA2" s="4" t="s">
-        <v>46</v>
+        <v>197</v>
       </c>
       <c r="AB2" s="4"/>
       <c r="AC2" s="5" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="AD2" s="6" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="AE2" s="5" t="s">
-        <v>58</v>
+        <v>48</v>
       </c>
       <c r="AF2" s="5" t="s">
-        <v>59</v>
+        <v>198</v>
       </c>
       <c r="AG2" s="7"/>
       <c r="AH2" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="AI2" s="4" t="s">
+        <v>202</v>
+      </c>
+      <c r="AJ2" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="AK2" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="AL2" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="AM2" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="AN2" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="AO2" s="8" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="3" spans="1:41" ht="27" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="B3" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="E3" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="F3" s="10"/>
+      <c r="G3" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="H3" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="AI2" s="4"/>
-      <c r="AJ2" s="7" t="s">
+      <c r="I3" s="11"/>
+      <c r="J3" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="AK2" s="5" t="s">
+      <c r="K3" s="11"/>
+      <c r="L3" s="12"/>
+      <c r="M3" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="AL2" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="AM2" s="5" t="s">
+      <c r="N3" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="AN2" s="5"/>
-      <c r="AO2" s="9" t="s">
+      <c r="O3" s="9" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="3" spans="1:41" ht="27" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="10" t="s">
+      <c r="P3" s="11"/>
+      <c r="Q3" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="B3" s="10" t="s">
+      <c r="R3" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="C3" s="10" t="s">
+      <c r="S3" s="12"/>
+      <c r="T3" s="12"/>
+      <c r="U3" s="12"/>
+      <c r="V3" s="13" t="s">
         <v>67</v>
       </c>
-      <c r="D3" s="10" t="s">
+      <c r="W3" s="13" t="s">
         <v>68</v>
       </c>
-      <c r="E3" s="10" t="s">
+      <c r="X3" s="13" t="s">
         <v>69</v>
       </c>
-      <c r="F3" s="11"/>
-      <c r="G3" s="10" t="s">
+      <c r="Y3" s="13" t="s">
         <v>70</v>
       </c>
-      <c r="H3" s="10" t="s">
+      <c r="Z3" s="11"/>
+      <c r="AA3" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="I3" s="12"/>
-      <c r="J3" s="10" t="s">
+      <c r="AB3" s="11"/>
+      <c r="AC3" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="K3" s="12"/>
-      <c r="L3" s="13"/>
-      <c r="M3" s="10" t="s">
+      <c r="AD3" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="N3" s="10" t="s">
+      <c r="AE3" s="11"/>
+      <c r="AF3" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="O3" s="10" t="s">
+      <c r="AG3" s="10"/>
+      <c r="AH3" s="9"/>
+      <c r="AI3" s="9"/>
+      <c r="AJ3" s="10"/>
+      <c r="AK3" s="10"/>
+      <c r="AL3" s="10"/>
+      <c r="AM3" s="9"/>
+      <c r="AN3" s="9"/>
+    </row>
+    <row r="4" spans="1:41" ht="27" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="9" t="s">
         <v>75</v>
       </c>
-      <c r="P3" s="12"/>
-      <c r="Q3" s="10" t="s">
+      <c r="B4" s="12"/>
+      <c r="C4" s="12"/>
+      <c r="D4" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="R3" s="10" t="s">
+      <c r="E4" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="S3" s="13"/>
-      <c r="T3" s="13"/>
-      <c r="U3" s="13"/>
-      <c r="V3" s="14" t="s">
+      <c r="F4" s="11"/>
+      <c r="G4" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="W3" s="14" t="s">
+      <c r="H4" s="9" t="s">
         <v>79</v>
       </c>
-      <c r="X3" s="14" t="s">
+      <c r="I4" s="11"/>
+      <c r="J4" s="9" t="s">
         <v>80</v>
       </c>
-      <c r="Y3" s="14" t="s">
+      <c r="K4" s="11"/>
+      <c r="L4" s="12"/>
+      <c r="M4" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="Z3" s="12"/>
-      <c r="AA3" s="10" t="s">
+      <c r="N4" s="9" t="s">
         <v>82</v>
       </c>
-      <c r="AB3" s="12"/>
-      <c r="AC3" s="10" t="s">
+      <c r="O4" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="AD3" s="10" t="s">
+      <c r="P4" s="11"/>
+      <c r="Q4" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="AE3" s="12"/>
-      <c r="AF3" s="10" t="s">
+      <c r="R4" s="9" t="s">
         <v>85</v>
       </c>
-      <c r="AG3" s="11"/>
-      <c r="AH3" s="10"/>
-      <c r="AI3" s="10"/>
-      <c r="AJ3" s="11"/>
-      <c r="AK3" s="11"/>
-      <c r="AL3" s="11"/>
-      <c r="AM3" s="10"/>
-      <c r="AN3" s="10"/>
-    </row>
-    <row r="4" spans="1:41" ht="27" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="10" t="s">
+      <c r="S4" s="12"/>
+      <c r="T4" s="12"/>
+      <c r="U4" s="12"/>
+      <c r="V4" s="13" t="s">
         <v>86</v>
       </c>
-      <c r="B4" s="13"/>
-      <c r="C4" s="13"/>
-      <c r="D4" s="10" t="s">
+      <c r="W4" s="12"/>
+      <c r="X4" s="13" t="s">
         <v>87</v>
       </c>
-      <c r="E4" s="10" t="s">
+      <c r="Y4" s="13" t="s">
         <v>88</v>
       </c>
-      <c r="F4" s="12"/>
-      <c r="G4" s="10" t="s">
+      <c r="Z4" s="11"/>
+      <c r="AA4" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="H4" s="10" t="s">
+      <c r="AB4" s="11"/>
+      <c r="AC4" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="I4" s="12"/>
-      <c r="J4" s="10" t="s">
+      <c r="AD4" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="K4" s="12"/>
-      <c r="L4" s="13"/>
-      <c r="M4" s="10" t="s">
+      <c r="AE4" s="11"/>
+      <c r="AF4" s="9" t="s">
         <v>92</v>
       </c>
-      <c r="N4" s="10" t="s">
+      <c r="AG4" s="10"/>
+      <c r="AH4" s="9"/>
+      <c r="AI4" s="9"/>
+      <c r="AJ4" s="10"/>
+      <c r="AK4" s="10"/>
+      <c r="AL4" s="10"/>
+      <c r="AM4" s="9"/>
+      <c r="AN4" s="9"/>
+    </row>
+    <row r="5" spans="1:41" ht="27" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="9" t="s">
         <v>93</v>
       </c>
-      <c r="O4" s="10" t="s">
+      <c r="B5" s="12"/>
+      <c r="C5" s="12"/>
+      <c r="D5" s="9" t="s">
         <v>94</v>
       </c>
-      <c r="P4" s="12"/>
-      <c r="Q4" s="10" t="s">
+      <c r="E5" s="9" t="s">
         <v>95</v>
       </c>
-      <c r="R4" s="10" t="s">
+      <c r="F5" s="11"/>
+      <c r="G5" s="12"/>
+      <c r="H5" s="9" t="s">
         <v>96</v>
       </c>
-      <c r="S4" s="13"/>
-      <c r="T4" s="13"/>
-      <c r="U4" s="13"/>
-      <c r="V4" s="14" t="s">
+      <c r="I5" s="11"/>
+      <c r="J5" s="9" t="s">
         <v>97</v>
       </c>
-      <c r="W4" s="13"/>
-      <c r="X4" s="14" t="s">
+      <c r="K5" s="11"/>
+      <c r="L5" s="12"/>
+      <c r="M5" s="9" t="s">
         <v>98</v>
       </c>
-      <c r="Y4" s="14" t="s">
+      <c r="N5" s="9" t="s">
         <v>99</v>
       </c>
-      <c r="Z4" s="12"/>
-      <c r="AA4" s="10" t="s">
+      <c r="O5" s="9" t="s">
         <v>100</v>
       </c>
-      <c r="AB4" s="12"/>
-      <c r="AC4" s="10" t="s">
+      <c r="P5" s="11"/>
+      <c r="Q5" s="9" t="s">
         <v>101</v>
       </c>
-      <c r="AD4" s="10" t="s">
+      <c r="R5" s="9" t="s">
         <v>102</v>
       </c>
-      <c r="AE4" s="12"/>
-      <c r="AF4" s="10" t="s">
+      <c r="S5" s="12"/>
+      <c r="T5" s="12"/>
+      <c r="U5" s="12"/>
+      <c r="V5" s="13" t="s">
         <v>103</v>
       </c>
-      <c r="AG4" s="11"/>
-      <c r="AH4" s="10"/>
-      <c r="AI4" s="10"/>
-      <c r="AJ4" s="11"/>
-      <c r="AK4" s="11"/>
-      <c r="AL4" s="11"/>
-      <c r="AM4" s="10"/>
-      <c r="AN4" s="10"/>
-    </row>
-    <row r="5" spans="1:41" ht="27" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="10" t="s">
+      <c r="W5" s="12"/>
+      <c r="X5" s="12"/>
+      <c r="Y5" s="13" t="s">
         <v>104</v>
       </c>
-      <c r="B5" s="13"/>
-      <c r="C5" s="13"/>
-      <c r="D5" s="10" t="s">
+      <c r="Z5" s="11"/>
+      <c r="AA5" s="9" t="s">
         <v>105</v>
       </c>
-      <c r="E5" s="10" t="s">
+      <c r="AB5" s="11"/>
+      <c r="AC5" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="F5" s="12"/>
-      <c r="G5" s="13"/>
-      <c r="H5" s="10" t="s">
+      <c r="AD5" s="12"/>
+      <c r="AE5" s="11"/>
+      <c r="AF5" s="9" t="s">
         <v>107</v>
       </c>
-      <c r="I5" s="12"/>
-      <c r="J5" s="10" t="s">
+      <c r="AG5" s="10"/>
+      <c r="AH5" s="9"/>
+      <c r="AI5" s="9"/>
+      <c r="AJ5" s="10"/>
+      <c r="AK5" s="10"/>
+      <c r="AL5" s="10"/>
+      <c r="AM5" s="9"/>
+      <c r="AN5" s="9"/>
+    </row>
+    <row r="6" spans="1:41" ht="27" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="9" t="s">
         <v>108</v>
       </c>
-      <c r="K5" s="12"/>
-      <c r="L5" s="13"/>
-      <c r="M5" s="10" t="s">
+      <c r="B6" s="12"/>
+      <c r="C6" s="12"/>
+      <c r="D6" s="9" t="s">
         <v>109</v>
       </c>
-      <c r="N5" s="10" t="s">
+      <c r="E6" s="9" t="s">
         <v>110</v>
       </c>
-      <c r="O5" s="10" t="s">
+      <c r="F6" s="11"/>
+      <c r="G6" s="12"/>
+      <c r="H6" s="9" t="s">
         <v>111</v>
       </c>
-      <c r="P5" s="12"/>
-      <c r="Q5" s="10" t="s">
+      <c r="I6" s="11"/>
+      <c r="J6" s="9" t="s">
         <v>112</v>
       </c>
-      <c r="R5" s="10" t="s">
+      <c r="K6" s="11"/>
+      <c r="L6" s="12"/>
+      <c r="M6" s="9" t="s">
         <v>113</v>
       </c>
-      <c r="S5" s="13"/>
-      <c r="T5" s="13"/>
-      <c r="U5" s="13"/>
-      <c r="V5" s="14" t="s">
+      <c r="N6" s="12"/>
+      <c r="O6" s="12"/>
+      <c r="P6" s="11"/>
+      <c r="Q6" s="9" t="s">
         <v>114</v>
       </c>
-      <c r="W5" s="13"/>
-      <c r="X5" s="13"/>
-      <c r="Y5" s="14" t="s">
+      <c r="R6" s="9" t="s">
         <v>115</v>
       </c>
-      <c r="Z5" s="12"/>
-      <c r="AA5" s="10" t="s">
+      <c r="S6" s="12"/>
+      <c r="T6" s="12"/>
+      <c r="U6" s="12"/>
+      <c r="V6" s="13" t="s">
         <v>116</v>
       </c>
-      <c r="AB5" s="12"/>
-      <c r="AC5" s="10" t="s">
+      <c r="W6" s="13" t="s">
         <v>117</v>
       </c>
-      <c r="AD5" s="13"/>
-      <c r="AE5" s="12"/>
-      <c r="AF5" s="10" t="s">
+      <c r="X6" s="12"/>
+      <c r="Y6" s="13" t="s">
         <v>118</v>
       </c>
-      <c r="AG5" s="11"/>
-      <c r="AH5" s="10"/>
-      <c r="AI5" s="10"/>
-      <c r="AJ5" s="11"/>
-      <c r="AK5" s="11"/>
-      <c r="AL5" s="11"/>
-      <c r="AM5" s="10"/>
-      <c r="AN5" s="10"/>
-    </row>
-    <row r="6" spans="1:41" ht="27" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="10" t="s">
+      <c r="Z6" s="11"/>
+      <c r="AA6" s="9" t="s">
         <v>119</v>
       </c>
-      <c r="B6" s="13"/>
-      <c r="C6" s="13"/>
-      <c r="D6" s="10" t="s">
+      <c r="AB6" s="11"/>
+      <c r="AC6" s="9" t="s">
         <v>120</v>
       </c>
-      <c r="E6" s="10" t="s">
+      <c r="AD6" s="12"/>
+      <c r="AE6" s="11"/>
+      <c r="AF6" s="9" t="s">
         <v>121</v>
       </c>
-      <c r="F6" s="12"/>
-      <c r="G6" s="13"/>
-      <c r="H6" s="10" t="s">
+      <c r="AG6" s="10"/>
+      <c r="AH6" s="9"/>
+      <c r="AI6" s="9"/>
+      <c r="AJ6" s="10"/>
+      <c r="AK6" s="10"/>
+      <c r="AL6" s="10"/>
+      <c r="AM6" s="9"/>
+      <c r="AN6" s="9"/>
+    </row>
+    <row r="7" spans="1:41" ht="27" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="9" t="s">
         <v>122</v>
       </c>
-      <c r="I6" s="12"/>
-      <c r="J6" s="10" t="s">
+      <c r="B7" s="12"/>
+      <c r="C7" s="12"/>
+      <c r="D7" s="9" t="s">
         <v>123</v>
       </c>
-      <c r="K6" s="12"/>
-      <c r="L6" s="13"/>
-      <c r="M6" s="10" t="s">
+      <c r="E7" s="9" t="s">
         <v>124</v>
       </c>
-      <c r="N6" s="13"/>
-      <c r="O6" s="13"/>
-      <c r="P6" s="12"/>
-      <c r="Q6" s="10" t="s">
+      <c r="F7" s="11"/>
+      <c r="G7" s="12"/>
+      <c r="H7" s="9" t="s">
         <v>125</v>
       </c>
-      <c r="R6" s="10" t="s">
+      <c r="I7" s="11"/>
+      <c r="J7" s="9" t="s">
         <v>126</v>
       </c>
-      <c r="S6" s="13"/>
-      <c r="T6" s="13"/>
-      <c r="U6" s="13"/>
-      <c r="V6" s="14" t="s">
+      <c r="K7" s="11"/>
+      <c r="L7" s="12"/>
+      <c r="M7" s="9" t="s">
         <v>127</v>
       </c>
-      <c r="W6" s="14" t="s">
+      <c r="N7" s="12"/>
+      <c r="O7" s="12"/>
+      <c r="P7" s="11"/>
+      <c r="Q7" s="9" t="s">
         <v>128</v>
       </c>
-      <c r="X6" s="13"/>
-      <c r="Y6" s="14" t="s">
+      <c r="R7" s="9" t="s">
         <v>129</v>
       </c>
-      <c r="Z6" s="12"/>
-      <c r="AA6" s="10" t="s">
+      <c r="S7" s="12"/>
+      <c r="T7" s="12"/>
+      <c r="U7" s="12"/>
+      <c r="V7" s="13" t="s">
         <v>130</v>
       </c>
-      <c r="AB6" s="12"/>
-      <c r="AC6" s="10" t="s">
+      <c r="W7" s="12"/>
+      <c r="X7" s="12"/>
+      <c r="Y7" s="11"/>
+      <c r="Z7" s="11"/>
+      <c r="AA7" s="9" t="s">
         <v>131</v>
       </c>
-      <c r="AD6" s="13"/>
-      <c r="AE6" s="12"/>
-      <c r="AF6" s="10" t="s">
+      <c r="AB7" s="11"/>
+      <c r="AC7" s="9" t="s">
         <v>132</v>
       </c>
-      <c r="AG6" s="11"/>
-      <c r="AH6" s="10"/>
-      <c r="AI6" s="10"/>
-      <c r="AJ6" s="11"/>
-      <c r="AK6" s="11"/>
-      <c r="AL6" s="11"/>
-      <c r="AM6" s="10"/>
-      <c r="AN6" s="10"/>
-    </row>
-    <row r="7" spans="1:41" ht="27" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="10" t="s">
+      <c r="AD7" s="12"/>
+      <c r="AE7" s="11"/>
+      <c r="AF7" s="9" t="s">
         <v>133</v>
       </c>
-      <c r="B7" s="13"/>
-      <c r="C7" s="13"/>
-      <c r="D7" s="10" t="s">
+      <c r="AG7" s="10"/>
+      <c r="AH7" s="9"/>
+      <c r="AI7" s="9"/>
+      <c r="AJ7" s="10"/>
+      <c r="AK7" s="10"/>
+      <c r="AL7" s="10"/>
+      <c r="AM7" s="9"/>
+      <c r="AN7" s="9"/>
+    </row>
+    <row r="8" spans="1:41" ht="27" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="9" t="s">
         <v>134</v>
       </c>
-      <c r="E7" s="10" t="s">
+      <c r="B8" s="12"/>
+      <c r="C8" s="12"/>
+      <c r="D8" s="12"/>
+      <c r="E8" s="9" t="s">
         <v>135</v>
       </c>
-      <c r="F7" s="12"/>
-      <c r="G7" s="13"/>
-      <c r="H7" s="10" t="s">
+      <c r="F8" s="11"/>
+      <c r="G8" s="12"/>
+      <c r="H8" s="12"/>
+      <c r="I8" s="11"/>
+      <c r="J8" s="12"/>
+      <c r="K8" s="11"/>
+      <c r="L8" s="12"/>
+      <c r="M8" s="9" t="s">
         <v>136</v>
       </c>
-      <c r="I7" s="12"/>
-      <c r="J7" s="10" t="s">
+      <c r="N8" s="12"/>
+      <c r="O8" s="12"/>
+      <c r="P8" s="11"/>
+      <c r="Q8" s="9" t="s">
         <v>137</v>
       </c>
-      <c r="K7" s="12"/>
-      <c r="L7" s="13"/>
-      <c r="M7" s="10" t="s">
+      <c r="R8" s="9" t="s">
         <v>138</v>
       </c>
-      <c r="N7" s="13"/>
-      <c r="O7" s="13"/>
-      <c r="P7" s="12"/>
-      <c r="Q7" s="10" t="s">
+      <c r="S8" s="12"/>
+      <c r="T8" s="12"/>
+      <c r="U8" s="12"/>
+      <c r="V8" s="13" t="s">
         <v>139</v>
       </c>
-      <c r="R7" s="10" t="s">
+      <c r="W8" s="13" t="s">
         <v>140</v>
       </c>
-      <c r="S7" s="13"/>
-      <c r="T7" s="13"/>
-      <c r="U7" s="13"/>
-      <c r="V7" s="14" t="s">
+      <c r="X8" s="12"/>
+      <c r="Y8" s="11"/>
+      <c r="Z8" s="11"/>
+      <c r="AA8" s="9" t="s">
         <v>141</v>
       </c>
-      <c r="W7" s="13"/>
-      <c r="X7" s="13"/>
-      <c r="Y7" s="12"/>
-      <c r="Z7" s="12"/>
-      <c r="AA7" s="10" t="s">
+      <c r="AB8" s="11"/>
+      <c r="AC8" s="9" t="s">
         <v>142</v>
       </c>
-      <c r="AB7" s="12"/>
-      <c r="AC7" s="10" t="s">
+      <c r="AD8" s="12"/>
+      <c r="AE8" s="11"/>
+      <c r="AF8" s="12"/>
+      <c r="AG8" s="10"/>
+      <c r="AH8" s="9"/>
+      <c r="AI8" s="9"/>
+      <c r="AJ8" s="10"/>
+      <c r="AK8" s="10"/>
+      <c r="AL8" s="10"/>
+      <c r="AM8" s="9"/>
+      <c r="AN8" s="9"/>
+    </row>
+    <row r="9" spans="1:41" ht="27" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="9" t="s">
         <v>143</v>
       </c>
-      <c r="AD7" s="13"/>
-      <c r="AE7" s="12"/>
-      <c r="AF7" s="10" t="s">
+      <c r="B9" s="12"/>
+      <c r="C9" s="12"/>
+      <c r="D9" s="12"/>
+      <c r="E9" s="9" t="s">
         <v>144</v>
       </c>
-      <c r="AG7" s="11"/>
-      <c r="AH7" s="10"/>
-      <c r="AI7" s="10"/>
-      <c r="AJ7" s="11"/>
-      <c r="AK7" s="11"/>
-      <c r="AL7" s="11"/>
-      <c r="AM7" s="10"/>
-      <c r="AN7" s="10"/>
-    </row>
-    <row r="8" spans="1:41" ht="27" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="10" t="s">
+      <c r="F9" s="11"/>
+      <c r="G9" s="12"/>
+      <c r="H9" s="12"/>
+      <c r="I9" s="11"/>
+      <c r="J9" s="12"/>
+      <c r="K9" s="11"/>
+      <c r="L9" s="12"/>
+      <c r="M9" s="9" t="s">
         <v>145</v>
       </c>
-      <c r="B8" s="13"/>
-      <c r="C8" s="13"/>
-      <c r="D8" s="13"/>
-      <c r="E8" s="10" t="s">
+      <c r="N9" s="12"/>
+      <c r="O9" s="12"/>
+      <c r="P9" s="11"/>
+      <c r="Q9" s="9" t="s">
         <v>146</v>
       </c>
-      <c r="F8" s="12"/>
-      <c r="G8" s="13"/>
-      <c r="H8" s="13"/>
-      <c r="I8" s="12"/>
-      <c r="J8" s="13"/>
-      <c r="K8" s="12"/>
-      <c r="L8" s="13"/>
-      <c r="M8" s="10" t="s">
+      <c r="R9" s="9" t="s">
         <v>147</v>
       </c>
-      <c r="N8" s="13"/>
-      <c r="O8" s="13"/>
-      <c r="P8" s="12"/>
-      <c r="Q8" s="10" t="s">
+      <c r="S9" s="12"/>
+      <c r="T9" s="12"/>
+      <c r="U9" s="12"/>
+      <c r="V9" s="13" t="s">
         <v>148</v>
       </c>
-      <c r="R8" s="10" t="s">
+      <c r="W9" s="13" t="s">
         <v>149</v>
       </c>
-      <c r="S8" s="13"/>
-      <c r="T8" s="13"/>
-      <c r="U8" s="13"/>
-      <c r="V8" s="14" t="s">
+      <c r="X9" s="12"/>
+      <c r="Y9" s="11"/>
+      <c r="Z9" s="11"/>
+      <c r="AA9" s="12"/>
+      <c r="AB9" s="11"/>
+      <c r="AC9" s="9" t="s">
         <v>150</v>
       </c>
-      <c r="W8" s="14" t="s">
+      <c r="AD9" s="12"/>
+      <c r="AE9" s="11"/>
+      <c r="AF9" s="12"/>
+      <c r="AG9" s="10"/>
+      <c r="AH9" s="9"/>
+      <c r="AI9" s="9"/>
+      <c r="AJ9" s="10"/>
+      <c r="AK9" s="10"/>
+      <c r="AL9" s="10"/>
+      <c r="AM9" s="9"/>
+      <c r="AN9" s="9"/>
+    </row>
+    <row r="10" spans="1:41" ht="27" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="9" t="s">
         <v>151</v>
       </c>
-      <c r="X8" s="13"/>
-      <c r="Y8" s="12"/>
-      <c r="Z8" s="12"/>
-      <c r="AA8" s="10" t="s">
+      <c r="B10" s="12"/>
+      <c r="C10" s="12"/>
+      <c r="D10" s="12"/>
+      <c r="E10" s="9" t="s">
         <v>152</v>
       </c>
-      <c r="AB8" s="12"/>
-      <c r="AC8" s="10" t="s">
+      <c r="F10" s="11"/>
+      <c r="G10" s="12"/>
+      <c r="H10" s="12"/>
+      <c r="I10" s="11"/>
+      <c r="J10" s="12"/>
+      <c r="K10" s="11"/>
+      <c r="L10" s="12"/>
+      <c r="M10" s="9" t="s">
         <v>153</v>
       </c>
-      <c r="AD8" s="13"/>
-      <c r="AE8" s="12"/>
-      <c r="AF8" s="13"/>
-      <c r="AG8" s="11"/>
-      <c r="AH8" s="10"/>
-      <c r="AI8" s="10"/>
-      <c r="AJ8" s="11"/>
-      <c r="AK8" s="11"/>
-      <c r="AL8" s="11"/>
-      <c r="AM8" s="10"/>
-      <c r="AN8" s="10"/>
-    </row>
-    <row r="9" spans="1:41" ht="27" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="10" t="s">
+      <c r="N10" s="12"/>
+      <c r="O10" s="12"/>
+      <c r="P10" s="11"/>
+      <c r="Q10" s="9" t="s">
         <v>154</v>
       </c>
-      <c r="B9" s="13"/>
-      <c r="C9" s="13"/>
-      <c r="D9" s="13"/>
-      <c r="E9" s="10" t="s">
+      <c r="R10" s="9" t="s">
         <v>155</v>
       </c>
-      <c r="F9" s="12"/>
-      <c r="G9" s="13"/>
-      <c r="H9" s="13"/>
-      <c r="I9" s="12"/>
-      <c r="J9" s="13"/>
-      <c r="K9" s="12"/>
-      <c r="L9" s="13"/>
-      <c r="M9" s="10" t="s">
+      <c r="S10" s="12"/>
+      <c r="T10" s="12"/>
+      <c r="U10" s="12"/>
+      <c r="V10" s="13"/>
+      <c r="W10" s="13" t="s">
         <v>156</v>
       </c>
-      <c r="N9" s="13"/>
-      <c r="O9" s="13"/>
-      <c r="P9" s="12"/>
-      <c r="Q9" s="10" t="s">
+      <c r="X10" s="12"/>
+      <c r="Y10" s="14"/>
+      <c r="Z10" s="11"/>
+      <c r="AA10" s="12"/>
+      <c r="AB10" s="11"/>
+      <c r="AC10" s="12"/>
+      <c r="AD10" s="12"/>
+      <c r="AE10" s="11"/>
+      <c r="AF10" s="12"/>
+      <c r="AG10" s="10"/>
+      <c r="AH10" s="9"/>
+      <c r="AI10" s="9"/>
+      <c r="AJ10" s="10"/>
+      <c r="AK10" s="10"/>
+      <c r="AL10" s="10"/>
+      <c r="AM10" s="9"/>
+      <c r="AN10" s="9"/>
+    </row>
+    <row r="11" spans="1:41" ht="27" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="9" t="s">
         <v>157</v>
       </c>
-      <c r="R9" s="10" t="s">
+      <c r="B11" s="12"/>
+      <c r="C11" s="12"/>
+      <c r="D11" s="12"/>
+      <c r="E11" s="9" t="s">
         <v>158</v>
       </c>
-      <c r="S9" s="13"/>
-      <c r="T9" s="13"/>
-      <c r="U9" s="13"/>
-      <c r="V9" s="14" t="s">
+      <c r="F11" s="11"/>
+      <c r="G11" s="12"/>
+      <c r="H11" s="12"/>
+      <c r="I11" s="11"/>
+      <c r="J11" s="12"/>
+      <c r="K11" s="11"/>
+      <c r="L11" s="12"/>
+      <c r="M11" s="12"/>
+      <c r="N11" s="12"/>
+      <c r="O11" s="12"/>
+      <c r="P11" s="11"/>
+      <c r="Q11" s="9" t="s">
         <v>159</v>
       </c>
-      <c r="W9" s="14" t="s">
+      <c r="R11" s="9" t="s">
         <v>160</v>
       </c>
-      <c r="X9" s="13"/>
-      <c r="Y9" s="12"/>
-      <c r="Z9" s="12"/>
-      <c r="AA9" s="13"/>
-      <c r="AB9" s="12"/>
-      <c r="AC9" s="10" t="s">
+      <c r="S11" s="12"/>
+      <c r="T11" s="12"/>
+      <c r="U11" s="12"/>
+      <c r="V11" s="13"/>
+      <c r="W11" s="13" t="s">
         <v>161</v>
       </c>
-      <c r="AD9" s="13"/>
-      <c r="AE9" s="12"/>
-      <c r="AF9" s="13"/>
-      <c r="AG9" s="11"/>
-      <c r="AH9" s="10"/>
-      <c r="AI9" s="10"/>
-      <c r="AJ9" s="11"/>
-      <c r="AK9" s="11"/>
-      <c r="AL9" s="11"/>
-      <c r="AM9" s="10"/>
-      <c r="AN9" s="10"/>
-    </row>
-    <row r="10" spans="1:41" ht="27" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="10" t="s">
+      <c r="X11" s="12"/>
+      <c r="Y11" s="11"/>
+      <c r="Z11" s="11"/>
+      <c r="AA11" s="12"/>
+      <c r="AB11" s="11"/>
+      <c r="AC11" s="12"/>
+      <c r="AD11" s="12"/>
+      <c r="AE11" s="11"/>
+      <c r="AF11" s="12"/>
+      <c r="AG11" s="10"/>
+      <c r="AH11" s="9"/>
+      <c r="AI11" s="9"/>
+      <c r="AJ11" s="10"/>
+      <c r="AK11" s="10"/>
+      <c r="AL11" s="10"/>
+      <c r="AM11" s="9"/>
+      <c r="AN11" s="9"/>
+    </row>
+    <row r="12" spans="1:41" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="15"/>
+      <c r="B12" s="12"/>
+      <c r="C12" s="12"/>
+      <c r="D12" s="12"/>
+      <c r="E12" s="12"/>
+      <c r="F12" s="11"/>
+      <c r="G12" s="12"/>
+      <c r="H12" s="12"/>
+      <c r="I12" s="11"/>
+      <c r="J12" s="12"/>
+      <c r="K12" s="11"/>
+      <c r="L12" s="12"/>
+      <c r="M12" s="12"/>
+      <c r="N12" s="12"/>
+      <c r="O12" s="12"/>
+      <c r="P12" s="11"/>
+      <c r="Q12" s="9" t="s">
         <v>162</v>
       </c>
-      <c r="B10" s="13"/>
-      <c r="C10" s="13"/>
-      <c r="D10" s="13"/>
-      <c r="E10" s="10" t="s">
+      <c r="R12" s="12"/>
+      <c r="S12" s="12"/>
+      <c r="T12" s="12"/>
+      <c r="U12" s="12"/>
+      <c r="V12" s="13"/>
+      <c r="W12" s="13" t="s">
         <v>163</v>
       </c>
-      <c r="F10" s="12"/>
-      <c r="G10" s="13"/>
-      <c r="H10" s="13"/>
-      <c r="I10" s="12"/>
-      <c r="J10" s="13"/>
-      <c r="K10" s="12"/>
-      <c r="L10" s="13"/>
-      <c r="M10" s="10" t="s">
+      <c r="X12" s="12"/>
+      <c r="Y12" s="12"/>
+      <c r="Z12" s="12"/>
+      <c r="AA12" s="12"/>
+      <c r="AB12" s="12"/>
+      <c r="AC12" s="12"/>
+      <c r="AD12" s="12"/>
+      <c r="AE12" s="12"/>
+      <c r="AF12" s="12"/>
+      <c r="AG12" s="9"/>
+      <c r="AH12" s="9"/>
+      <c r="AI12" s="9"/>
+      <c r="AJ12" s="9"/>
+      <c r="AK12" s="9"/>
+      <c r="AL12" s="9"/>
+      <c r="AM12" s="9"/>
+      <c r="AN12" s="9"/>
+    </row>
+    <row r="13" spans="1:41" x14ac:dyDescent="0.3">
+      <c r="A13" s="12"/>
+      <c r="B13" s="12"/>
+      <c r="C13" s="12"/>
+      <c r="D13" s="12"/>
+      <c r="E13" s="12"/>
+      <c r="F13" s="11"/>
+      <c r="G13" s="12"/>
+      <c r="H13" s="12"/>
+      <c r="I13" s="11"/>
+      <c r="J13" s="12"/>
+      <c r="K13" s="11"/>
+      <c r="L13" s="12"/>
+      <c r="M13" s="12"/>
+      <c r="N13" s="12"/>
+      <c r="O13" s="12"/>
+      <c r="P13" s="11"/>
+      <c r="Q13" s="12"/>
+      <c r="R13" s="12"/>
+      <c r="S13" s="12"/>
+      <c r="T13" s="12"/>
+      <c r="U13" s="12"/>
+      <c r="V13" s="13"/>
+      <c r="W13" s="12"/>
+      <c r="X13" s="12"/>
+      <c r="Y13" s="12"/>
+      <c r="Z13" s="12"/>
+      <c r="AA13" s="12"/>
+      <c r="AB13" s="12"/>
+      <c r="AC13" s="12"/>
+      <c r="AD13" s="12"/>
+      <c r="AE13" s="12"/>
+      <c r="AF13" s="12"/>
+      <c r="AG13" s="9"/>
+      <c r="AH13" s="9"/>
+      <c r="AI13" s="9"/>
+      <c r="AJ13" s="9"/>
+      <c r="AK13" s="9"/>
+      <c r="AL13" s="9"/>
+      <c r="AM13" s="9"/>
+      <c r="AN13" s="9"/>
+    </row>
+    <row r="14" spans="1:41" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="12"/>
+      <c r="B14" s="12"/>
+      <c r="C14" s="12"/>
+      <c r="D14" s="12"/>
+      <c r="E14" s="12"/>
+      <c r="F14" s="11"/>
+      <c r="G14" s="12"/>
+      <c r="H14" s="12"/>
+      <c r="I14" s="11"/>
+      <c r="J14" s="12"/>
+      <c r="K14" s="11"/>
+      <c r="L14" s="12"/>
+      <c r="M14" s="12"/>
+      <c r="N14" s="12"/>
+      <c r="O14" s="12"/>
+      <c r="P14" s="11"/>
+      <c r="Q14" s="12"/>
+      <c r="R14" s="12"/>
+      <c r="S14" s="12"/>
+      <c r="T14" s="12"/>
+      <c r="U14" s="12"/>
+      <c r="V14" s="13"/>
+      <c r="W14" s="13" t="s">
         <v>164</v>
       </c>
-      <c r="N10" s="13"/>
-      <c r="O10" s="13"/>
-      <c r="P10" s="12"/>
-      <c r="Q10" s="10" t="s">
+      <c r="X14" s="12"/>
+      <c r="Y14" s="12"/>
+      <c r="Z14" s="12"/>
+      <c r="AA14" s="12"/>
+      <c r="AB14" s="12"/>
+      <c r="AC14" s="12"/>
+      <c r="AD14" s="12"/>
+      <c r="AE14" s="12"/>
+      <c r="AF14" s="12"/>
+      <c r="AG14" s="9"/>
+      <c r="AH14" s="9"/>
+      <c r="AI14" s="9"/>
+      <c r="AJ14" s="9"/>
+      <c r="AK14" s="9"/>
+      <c r="AL14" s="9"/>
+      <c r="AM14" s="9"/>
+      <c r="AN14" s="9"/>
+    </row>
+    <row r="15" spans="1:41" x14ac:dyDescent="0.3">
+      <c r="A15" s="12"/>
+      <c r="B15" s="12"/>
+      <c r="C15" s="12"/>
+      <c r="D15" s="12"/>
+      <c r="E15" s="12"/>
+      <c r="F15" s="12"/>
+      <c r="G15" s="12"/>
+      <c r="H15" s="12"/>
+      <c r="I15" s="12"/>
+      <c r="J15" s="12"/>
+      <c r="K15" s="12"/>
+      <c r="L15" s="12"/>
+      <c r="M15" s="12"/>
+      <c r="N15" s="12"/>
+      <c r="O15" s="12"/>
+      <c r="P15" s="12"/>
+      <c r="Q15" s="12"/>
+      <c r="R15" s="12"/>
+      <c r="S15" s="12"/>
+      <c r="T15" s="12"/>
+      <c r="U15" s="12"/>
+      <c r="V15" s="13"/>
+      <c r="W15" s="12"/>
+      <c r="X15" s="12"/>
+      <c r="Y15" s="12"/>
+      <c r="Z15" s="12"/>
+      <c r="AA15" s="12"/>
+      <c r="AB15" s="12"/>
+      <c r="AC15" s="12"/>
+      <c r="AD15" s="12"/>
+      <c r="AE15" s="12"/>
+      <c r="AF15" s="12"/>
+      <c r="AG15" s="9"/>
+      <c r="AH15" s="9"/>
+      <c r="AI15" s="9"/>
+      <c r="AJ15" s="9"/>
+      <c r="AK15" s="9"/>
+      <c r="AL15" s="9"/>
+      <c r="AM15" s="9"/>
+      <c r="AN15" s="9"/>
+    </row>
+    <row r="16" spans="1:41" ht="27" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="12"/>
+      <c r="B16" s="12"/>
+      <c r="C16" s="12"/>
+      <c r="D16" s="12"/>
+      <c r="E16" s="12"/>
+      <c r="F16" s="12"/>
+      <c r="G16" s="12"/>
+      <c r="H16" s="12"/>
+      <c r="I16" s="12"/>
+      <c r="J16" s="12"/>
+      <c r="K16" s="12"/>
+      <c r="L16" s="12"/>
+      <c r="M16" s="12"/>
+      <c r="N16" s="12"/>
+      <c r="O16" s="12"/>
+      <c r="P16" s="12"/>
+      <c r="Q16" s="12"/>
+      <c r="R16" s="12"/>
+      <c r="S16" s="12"/>
+      <c r="T16" s="12"/>
+      <c r="U16" s="12"/>
+      <c r="V16" s="13"/>
+      <c r="W16" s="13" t="s">
         <v>165</v>
       </c>
-      <c r="R10" s="10" t="s">
-        <v>166</v>
-      </c>
-      <c r="S10" s="13"/>
-      <c r="T10" s="13"/>
-      <c r="U10" s="13"/>
-      <c r="V10" s="14"/>
-      <c r="W10" s="14" t="s">
-        <v>167</v>
-      </c>
-      <c r="X10" s="13"/>
-      <c r="Y10" s="15"/>
-      <c r="Z10" s="12"/>
-      <c r="AA10" s="13"/>
-      <c r="AB10" s="12"/>
-      <c r="AC10" s="13"/>
-      <c r="AD10" s="13"/>
-      <c r="AE10" s="12"/>
-      <c r="AF10" s="13"/>
-      <c r="AG10" s="11"/>
-      <c r="AH10" s="10"/>
-      <c r="AI10" s="10"/>
-      <c r="AJ10" s="11"/>
-      <c r="AK10" s="11"/>
-      <c r="AL10" s="11"/>
-      <c r="AM10" s="10"/>
-      <c r="AN10" s="10"/>
-    </row>
-    <row r="11" spans="1:41" ht="27" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="10" t="s">
-        <v>168</v>
-      </c>
-      <c r="B11" s="13"/>
-      <c r="C11" s="13"/>
-      <c r="D11" s="13"/>
-      <c r="E11" s="10" t="s">
-        <v>169</v>
-      </c>
-      <c r="F11" s="12"/>
-      <c r="G11" s="13"/>
-      <c r="H11" s="13"/>
-      <c r="I11" s="12"/>
-      <c r="J11" s="13"/>
-      <c r="K11" s="12"/>
-      <c r="L11" s="13"/>
-      <c r="M11" s="13"/>
-      <c r="N11" s="13"/>
-      <c r="O11" s="13"/>
-      <c r="P11" s="12"/>
-      <c r="Q11" s="10" t="s">
-        <v>170</v>
-      </c>
-      <c r="R11" s="10" t="s">
-        <v>171</v>
-      </c>
-      <c r="S11" s="13"/>
-      <c r="T11" s="13"/>
-      <c r="U11" s="13"/>
-      <c r="V11" s="14"/>
-      <c r="W11" s="14" t="s">
-        <v>172</v>
-      </c>
-      <c r="X11" s="13"/>
-      <c r="Y11" s="12"/>
-      <c r="Z11" s="12"/>
-      <c r="AA11" s="13"/>
-      <c r="AB11" s="12"/>
-      <c r="AC11" s="13"/>
-      <c r="AD11" s="13"/>
-      <c r="AE11" s="12"/>
-      <c r="AF11" s="13"/>
-      <c r="AG11" s="11"/>
-      <c r="AH11" s="10"/>
-      <c r="AI11" s="10"/>
-      <c r="AJ11" s="11"/>
-      <c r="AK11" s="11"/>
-      <c r="AL11" s="11"/>
-      <c r="AM11" s="10"/>
-      <c r="AN11" s="10"/>
-    </row>
-    <row r="12" spans="1:41" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="16"/>
-      <c r="B12" s="13"/>
-      <c r="C12" s="13"/>
-      <c r="D12" s="13"/>
-      <c r="E12" s="13"/>
-      <c r="F12" s="12"/>
-      <c r="G12" s="13"/>
-      <c r="H12" s="13"/>
-      <c r="I12" s="12"/>
-      <c r="J12" s="13"/>
-      <c r="K12" s="12"/>
-      <c r="L12" s="13"/>
-      <c r="M12" s="13"/>
-      <c r="N12" s="13"/>
-      <c r="O12" s="13"/>
-      <c r="P12" s="12"/>
-      <c r="Q12" s="10" t="s">
-        <v>173</v>
-      </c>
-      <c r="R12" s="13"/>
-      <c r="S12" s="13"/>
-      <c r="T12" s="13"/>
-      <c r="U12" s="13"/>
-      <c r="V12" s="14"/>
-      <c r="W12" s="14" t="s">
-        <v>174</v>
-      </c>
-      <c r="X12" s="13"/>
-      <c r="Y12" s="13"/>
-      <c r="Z12" s="13"/>
-      <c r="AA12" s="13"/>
-      <c r="AB12" s="13"/>
-      <c r="AC12" s="13"/>
-      <c r="AD12" s="13"/>
-      <c r="AE12" s="13"/>
-      <c r="AF12" s="13"/>
-      <c r="AG12" s="10"/>
-      <c r="AH12" s="10"/>
-      <c r="AI12" s="10"/>
-      <c r="AJ12" s="10"/>
-      <c r="AK12" s="10"/>
-      <c r="AL12" s="10"/>
-      <c r="AM12" s="10"/>
-      <c r="AN12" s="10"/>
-    </row>
-    <row r="13" spans="1:41" x14ac:dyDescent="0.3">
-      <c r="A13" s="13"/>
-      <c r="B13" s="13"/>
-      <c r="C13" s="13"/>
-      <c r="D13" s="13"/>
-      <c r="E13" s="13"/>
-      <c r="F13" s="12"/>
-      <c r="G13" s="13"/>
-      <c r="H13" s="13"/>
-      <c r="I13" s="12"/>
-      <c r="J13" s="13"/>
-      <c r="K13" s="12"/>
-      <c r="L13" s="13"/>
-      <c r="M13" s="13"/>
-      <c r="N13" s="13"/>
-      <c r="O13" s="13"/>
-      <c r="P13" s="12"/>
-      <c r="Q13" s="13"/>
-      <c r="R13" s="13"/>
-      <c r="S13" s="13"/>
-      <c r="T13" s="13"/>
-      <c r="U13" s="13"/>
-      <c r="V13" s="14"/>
-      <c r="W13" s="13"/>
-      <c r="X13" s="13"/>
-      <c r="Y13" s="13"/>
-      <c r="Z13" s="13"/>
-      <c r="AA13" s="13"/>
-      <c r="AB13" s="13"/>
-      <c r="AC13" s="13"/>
-      <c r="AD13" s="13"/>
-      <c r="AE13" s="13"/>
-      <c r="AF13" s="13"/>
-      <c r="AG13" s="10"/>
-      <c r="AH13" s="10"/>
-      <c r="AI13" s="10"/>
-      <c r="AJ13" s="10"/>
-      <c r="AK13" s="10"/>
-      <c r="AL13" s="10"/>
-      <c r="AM13" s="10"/>
-      <c r="AN13" s="10"/>
-    </row>
-    <row r="14" spans="1:41" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="13"/>
-      <c r="B14" s="13"/>
-      <c r="C14" s="13"/>
-      <c r="D14" s="13"/>
-      <c r="E14" s="13"/>
-      <c r="F14" s="12"/>
-      <c r="G14" s="13"/>
-      <c r="H14" s="13"/>
-      <c r="I14" s="12"/>
-      <c r="J14" s="13"/>
-      <c r="K14" s="12"/>
-      <c r="L14" s="13"/>
-      <c r="M14" s="13"/>
-      <c r="N14" s="13"/>
-      <c r="O14" s="13"/>
-      <c r="P14" s="12"/>
-      <c r="Q14" s="13"/>
-      <c r="R14" s="13"/>
-      <c r="S14" s="13"/>
-      <c r="T14" s="13"/>
-      <c r="U14" s="13"/>
-      <c r="V14" s="14"/>
-      <c r="W14" s="14" t="s">
-        <v>175</v>
-      </c>
-      <c r="X14" s="13"/>
-      <c r="Y14" s="13"/>
-      <c r="Z14" s="13"/>
-      <c r="AA14" s="13"/>
-      <c r="AB14" s="13"/>
-      <c r="AC14" s="13"/>
-      <c r="AD14" s="13"/>
-      <c r="AE14" s="13"/>
-      <c r="AF14" s="13"/>
-      <c r="AG14" s="10"/>
-      <c r="AH14" s="10"/>
-      <c r="AI14" s="10"/>
-      <c r="AJ14" s="10"/>
-      <c r="AK14" s="10"/>
-      <c r="AL14" s="10"/>
-      <c r="AM14" s="10"/>
-      <c r="AN14" s="10"/>
-    </row>
-    <row r="15" spans="1:41" x14ac:dyDescent="0.3">
-      <c r="A15" s="13"/>
-      <c r="B15" s="13"/>
-      <c r="C15" s="13"/>
-      <c r="D15" s="13"/>
-      <c r="E15" s="13"/>
-      <c r="F15" s="13"/>
-      <c r="G15" s="13"/>
-      <c r="H15" s="13"/>
-      <c r="I15" s="13"/>
-      <c r="J15" s="13"/>
-      <c r="K15" s="13"/>
-      <c r="L15" s="13"/>
-      <c r="M15" s="13"/>
-      <c r="N15" s="13"/>
-      <c r="O15" s="13"/>
-      <c r="P15" s="13"/>
-      <c r="Q15" s="13"/>
-      <c r="R15" s="13"/>
-      <c r="S15" s="13"/>
-      <c r="T15" s="13"/>
-      <c r="U15" s="13"/>
-      <c r="V15" s="14"/>
-      <c r="W15" s="13"/>
-      <c r="X15" s="13"/>
-      <c r="Y15" s="13"/>
-      <c r="Z15" s="13"/>
-      <c r="AA15" s="13"/>
-      <c r="AB15" s="13"/>
-      <c r="AC15" s="13"/>
-      <c r="AD15" s="13"/>
-      <c r="AE15" s="13"/>
-      <c r="AF15" s="13"/>
-      <c r="AG15" s="10"/>
-      <c r="AH15" s="10"/>
-      <c r="AI15" s="10"/>
-      <c r="AJ15" s="10"/>
-      <c r="AK15" s="10"/>
-      <c r="AL15" s="10"/>
-      <c r="AM15" s="10"/>
-      <c r="AN15" s="10"/>
-    </row>
-    <row r="16" spans="1:41" ht="27" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="13"/>
-      <c r="B16" s="13"/>
-      <c r="C16" s="13"/>
-      <c r="D16" s="13"/>
-      <c r="E16" s="13"/>
-      <c r="F16" s="13"/>
-      <c r="G16" s="13"/>
-      <c r="H16" s="13"/>
-      <c r="I16" s="13"/>
-      <c r="J16" s="13"/>
-      <c r="K16" s="13"/>
-      <c r="L16" s="13"/>
-      <c r="M16" s="13"/>
-      <c r="N16" s="13"/>
-      <c r="O16" s="13"/>
-      <c r="P16" s="13"/>
-      <c r="Q16" s="13"/>
-      <c r="R16" s="13"/>
-      <c r="S16" s="13"/>
-      <c r="T16" s="13"/>
-      <c r="U16" s="13"/>
-      <c r="V16" s="14"/>
-      <c r="W16" s="14" t="s">
-        <v>176</v>
-      </c>
-      <c r="X16" s="13"/>
-      <c r="Y16" s="13"/>
-      <c r="Z16" s="13"/>
-      <c r="AA16" s="13"/>
-      <c r="AB16" s="13"/>
-      <c r="AC16" s="13"/>
-      <c r="AD16" s="13"/>
-      <c r="AE16" s="13"/>
-      <c r="AF16" s="13"/>
-      <c r="AG16" s="10"/>
-      <c r="AH16" s="10"/>
-      <c r="AI16" s="10"/>
-      <c r="AJ16" s="10"/>
-      <c r="AK16" s="10"/>
-      <c r="AL16" s="10"/>
-      <c r="AM16" s="10"/>
-      <c r="AN16" s="10"/>
+      <c r="X16" s="12"/>
+      <c r="Y16" s="12"/>
+      <c r="Z16" s="12"/>
+      <c r="AA16" s="12"/>
+      <c r="AB16" s="12"/>
+      <c r="AC16" s="12"/>
+      <c r="AD16" s="12"/>
+      <c r="AE16" s="12"/>
+      <c r="AF16" s="12"/>
+      <c r="AG16" s="9"/>
+      <c r="AH16" s="9"/>
+      <c r="AI16" s="9"/>
+      <c r="AJ16" s="9"/>
+      <c r="AK16" s="9"/>
+      <c r="AL16" s="9"/>
+      <c r="AM16" s="9"/>
+      <c r="AN16" s="9"/>
     </row>
     <row r="17" spans="1:40" x14ac:dyDescent="0.3">
-      <c r="A17" s="13"/>
-      <c r="B17" s="13"/>
-      <c r="C17" s="13"/>
-      <c r="D17" s="13"/>
-      <c r="E17" s="13"/>
-      <c r="F17" s="13"/>
-      <c r="G17" s="13"/>
-      <c r="H17" s="13"/>
-      <c r="I17" s="13"/>
-      <c r="J17" s="13"/>
-      <c r="K17" s="13"/>
-      <c r="L17" s="13"/>
-      <c r="M17" s="13"/>
-      <c r="N17" s="13"/>
-      <c r="O17" s="13"/>
-      <c r="P17" s="13"/>
-      <c r="Q17" s="13"/>
-      <c r="R17" s="13"/>
-      <c r="S17" s="13"/>
-      <c r="T17" s="13"/>
-      <c r="U17" s="13"/>
-      <c r="V17" s="14"/>
-      <c r="W17" s="13"/>
-      <c r="X17" s="13"/>
-      <c r="Y17" s="13"/>
-      <c r="Z17" s="13"/>
-      <c r="AA17" s="13"/>
-      <c r="AB17" s="13"/>
-      <c r="AC17" s="13"/>
-      <c r="AD17" s="13"/>
-      <c r="AE17" s="13"/>
-      <c r="AF17" s="13"/>
-      <c r="AG17" s="10"/>
-      <c r="AH17" s="10"/>
-      <c r="AI17" s="10"/>
-      <c r="AJ17" s="10"/>
-      <c r="AK17" s="10"/>
-      <c r="AL17" s="10"/>
-      <c r="AM17" s="10"/>
-      <c r="AN17" s="10"/>
+      <c r="A17" s="12"/>
+      <c r="B17" s="12"/>
+      <c r="C17" s="12"/>
+      <c r="D17" s="12"/>
+      <c r="E17" s="12"/>
+      <c r="F17" s="12"/>
+      <c r="G17" s="12"/>
+      <c r="H17" s="12"/>
+      <c r="I17" s="12"/>
+      <c r="J17" s="12"/>
+      <c r="K17" s="12"/>
+      <c r="L17" s="12"/>
+      <c r="M17" s="12"/>
+      <c r="N17" s="12"/>
+      <c r="O17" s="12"/>
+      <c r="P17" s="12"/>
+      <c r="Q17" s="12"/>
+      <c r="R17" s="12"/>
+      <c r="S17" s="12"/>
+      <c r="T17" s="12"/>
+      <c r="U17" s="12"/>
+      <c r="V17" s="13"/>
+      <c r="W17" s="12"/>
+      <c r="X17" s="12"/>
+      <c r="Y17" s="12"/>
+      <c r="Z17" s="12"/>
+      <c r="AA17" s="12"/>
+      <c r="AB17" s="12"/>
+      <c r="AC17" s="12"/>
+      <c r="AD17" s="12"/>
+      <c r="AE17" s="12"/>
+      <c r="AF17" s="12"/>
+      <c r="AG17" s="9"/>
+      <c r="AH17" s="9"/>
+      <c r="AI17" s="9"/>
+      <c r="AJ17" s="9"/>
+      <c r="AK17" s="9"/>
+      <c r="AL17" s="9"/>
+      <c r="AM17" s="9"/>
+      <c r="AN17" s="9"/>
     </row>
     <row r="18" spans="1:40" x14ac:dyDescent="0.3">
-      <c r="A18" s="13"/>
-      <c r="B18" s="13"/>
-      <c r="C18" s="13"/>
-      <c r="D18" s="13"/>
-      <c r="E18" s="13"/>
-      <c r="F18" s="13"/>
-      <c r="G18" s="13"/>
-      <c r="H18" s="13"/>
-      <c r="I18" s="13"/>
-      <c r="J18" s="13"/>
-      <c r="K18" s="13"/>
-      <c r="L18" s="13"/>
-      <c r="M18" s="13"/>
-      <c r="N18" s="13"/>
-      <c r="O18" s="13"/>
-      <c r="P18" s="13"/>
-      <c r="Q18" s="13"/>
-      <c r="R18" s="13"/>
-      <c r="S18" s="13"/>
-      <c r="T18" s="13"/>
-      <c r="U18" s="13"/>
-      <c r="V18" s="14"/>
-      <c r="W18" s="13"/>
-      <c r="X18" s="13"/>
-      <c r="Y18" s="13"/>
-      <c r="Z18" s="13"/>
-      <c r="AA18" s="13"/>
-      <c r="AB18" s="13"/>
-      <c r="AC18" s="13"/>
-      <c r="AD18" s="13"/>
-      <c r="AE18" s="13"/>
-      <c r="AF18" s="13"/>
-      <c r="AG18" s="10"/>
-      <c r="AH18" s="10"/>
-      <c r="AI18" s="10"/>
-      <c r="AJ18" s="10"/>
-      <c r="AK18" s="10"/>
-      <c r="AL18" s="10"/>
-      <c r="AM18" s="10"/>
-      <c r="AN18" s="10"/>
+      <c r="A18" s="12"/>
+      <c r="B18" s="12"/>
+      <c r="C18" s="12"/>
+      <c r="D18" s="12"/>
+      <c r="E18" s="12"/>
+      <c r="F18" s="12"/>
+      <c r="G18" s="12"/>
+      <c r="H18" s="12"/>
+      <c r="I18" s="12"/>
+      <c r="J18" s="12"/>
+      <c r="K18" s="12"/>
+      <c r="L18" s="12"/>
+      <c r="M18" s="12"/>
+      <c r="N18" s="12"/>
+      <c r="O18" s="12"/>
+      <c r="P18" s="12"/>
+      <c r="Q18" s="12"/>
+      <c r="R18" s="12"/>
+      <c r="S18" s="12"/>
+      <c r="T18" s="12"/>
+      <c r="U18" s="12"/>
+      <c r="V18" s="13"/>
+      <c r="W18" s="12"/>
+      <c r="X18" s="12"/>
+      <c r="Y18" s="12"/>
+      <c r="Z18" s="12"/>
+      <c r="AA18" s="12"/>
+      <c r="AB18" s="12"/>
+      <c r="AC18" s="12"/>
+      <c r="AD18" s="12"/>
+      <c r="AE18" s="12"/>
+      <c r="AF18" s="12"/>
+      <c r="AG18" s="9"/>
+      <c r="AH18" s="9"/>
+      <c r="AI18" s="9"/>
+      <c r="AJ18" s="9"/>
+      <c r="AK18" s="9"/>
+      <c r="AL18" s="9"/>
+      <c r="AM18" s="9"/>
+      <c r="AN18" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2345,25 +2349,25 @@
   <sheetData>
     <row r="1" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>177</v>
+        <v>166</v>
       </c>
       <c r="B1" t="s">
-        <v>178</v>
+        <v>167</v>
       </c>
       <c r="C1" t="s">
-        <v>179</v>
+        <v>168</v>
       </c>
       <c r="D1" t="s">
-        <v>180</v>
+        <v>169</v>
       </c>
       <c r="E1" t="s">
-        <v>181</v>
+        <v>170</v>
       </c>
       <c r="F1" t="s">
-        <v>182</v>
+        <v>171</v>
       </c>
       <c r="G1" t="s">
-        <v>199</v>
+        <v>183</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -2371,22 +2375,22 @@
         <v>4119</v>
       </c>
       <c r="B2" t="s">
-        <v>198</v>
+        <v>182</v>
       </c>
       <c r="C2" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="D2" t="s">
+        <v>172</v>
+      </c>
+      <c r="E2" t="s">
+        <v>40</v>
+      </c>
+      <c r="F2" s="16" t="s">
+        <v>173</v>
+      </c>
+      <c r="G2" t="s">
         <v>184</v>
-      </c>
-      <c r="E2" t="s">
-        <v>43</v>
-      </c>
-      <c r="F2" s="17" t="s">
-        <v>185</v>
-      </c>
-      <c r="G2" t="s">
-        <v>200</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
@@ -2394,19 +2398,19 @@
         <v>4120</v>
       </c>
       <c r="B3" t="s">
-        <v>186</v>
+        <v>174</v>
       </c>
       <c r="C3" t="s">
         <v>187</v>
       </c>
       <c r="D3" t="s">
-        <v>188</v>
+        <v>175</v>
       </c>
       <c r="E3" t="s">
-        <v>189</v>
-      </c>
-      <c r="F3" s="17" t="s">
-        <v>190</v>
+        <v>176</v>
+      </c>
+      <c r="F3" s="16" t="s">
+        <v>177</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
@@ -2414,16 +2418,16 @@
         <v>4121</v>
       </c>
       <c r="C4" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="D4" t="s">
-        <v>192</v>
+        <v>178</v>
       </c>
       <c r="E4" t="s">
-        <v>193</v>
-      </c>
-      <c r="F4" s="17" t="s">
-        <v>194</v>
+        <v>179</v>
+      </c>
+      <c r="F4" s="16" t="s">
+        <v>180</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
@@ -2431,10 +2435,10 @@
         <v>4122</v>
       </c>
       <c r="C5" t="s">
-        <v>195</v>
+        <v>189</v>
       </c>
       <c r="D5" t="s">
-        <v>196</v>
+        <v>181</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="27" customHeight="1" x14ac:dyDescent="0.3">
@@ -2442,7 +2446,7 @@
         <v>4123</v>
       </c>
       <c r="C6" t="s">
-        <v>197</v>
+        <v>186</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="27" customHeight="1" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Fix: HBR indirme formatı - MIME type Excel olarak ayarlandı (.htm yerine .xlsx)
</commit_message>
<xml_diff>
--- a/data/kocaeli/Veriler.xlsx
+++ b/data/kocaeli/Veriler.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fatiherkin\Desktop\bozankaya_ssh_takip\data\kocaeli\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7844EDDC-B026-4A43-AD8D-4F905FB6576E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22FE2DA0-BB5D-4AD2-8F61-7B015E565403}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2475,19 +2475,29 @@
       </c>
     </row>
     <row r="12" spans="1:7" ht="27" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="1"/>
+      <c r="A12" s="1">
+        <v>4129</v>
+      </c>
     </row>
     <row r="13" spans="1:7" ht="27" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="1"/>
+      <c r="A13" s="1">
+        <v>4130</v>
+      </c>
     </row>
     <row r="14" spans="1:7" ht="27" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="1"/>
+      <c r="A14" s="1">
+        <v>4131</v>
+      </c>
     </row>
     <row r="15" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="1"/>
+      <c r="A15" s="1">
+        <v>4132</v>
+      </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A16" s="1"/>
+      <c r="A16" s="1">
+        <v>4133</v>
+      </c>
     </row>
     <row r="17" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1"/>

</xml_diff>

<commit_message>
FRACAS modal formu - tüm dinamik dropdown alanları eklendi (sistem, alt_sistem, tedarikçi, arıza_sınıfı, kaynağı, tipi)
</commit_message>
<xml_diff>
--- a/data/kocaeli/Veriler.xlsx
+++ b/data/kocaeli/Veriler.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fatiherkin\Desktop\bozankaya_ssh_takip\data\kocaeli\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2C354E5-29E3-4D46-9700-E6EA47456AE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36D3DB65-8A9C-4B07-9E34-D5A36C2ACC12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1536" yWindow="1536" windowWidth="17280" windowHeight="9960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sayfa1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="204">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="205">
   <si>
     <t>Traction_Converter</t>
   </si>
@@ -646,6 +646,9 @@
   </si>
   <si>
     <t>ISRI</t>
+  </si>
+  <si>
+    <t>KAPI ÜSTÜ EKRAN</t>
   </si>
 </sst>
 </file>
@@ -1566,7 +1569,9 @@
       <c r="V4" s="13" t="s">
         <v>86</v>
       </c>
-      <c r="W4" s="12"/>
+      <c r="W4" s="13" t="s">
+        <v>204</v>
+      </c>
       <c r="X4" s="13" t="s">
         <v>87</v>
       </c>
@@ -2475,29 +2480,19 @@
       </c>
     </row>
     <row r="12" spans="1:7" ht="27" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="1">
-        <v>4129</v>
-      </c>
+      <c r="A12" s="1"/>
     </row>
     <row r="13" spans="1:7" ht="27" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="1">
-        <v>4130</v>
-      </c>
+      <c r="A13" s="1"/>
     </row>
     <row r="14" spans="1:7" ht="27" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="1">
-        <v>4131</v>
-      </c>
+      <c r="A14" s="1"/>
     </row>
     <row r="15" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="1">
-        <v>4132</v>
-      </c>
+      <c r="A15" s="1"/>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A16" s="1">
-        <v>4133</v>
-      </c>
+      <c r="A16" s="1"/>
     </row>
     <row r="17" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1"/>

</xml_diff>